<commit_message>
fix(ci): make E13 test-link a symbol-aware ratchet (fixes whole-repo FAIL)
</commit_message>
<xml_diff>
--- a/docs/build-provenance/PROMPT_MASTER_LOG.xlsx
+++ b/docs/build-provenance/PROMPT_MASTER_LOG.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roster Index" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prompt Chain'!$A$1:$S$106</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prompt Chain'!$A$1:$S$113</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -491,7 +491,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S106"/>
+  <dimension ref="A1:S113"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -10019,8 +10019,645 @@
         </is>
       </c>
     </row>
+    <row r="107">
+      <c r="A107" s="6" t="n">
+        <v>106</v>
+      </c>
+      <c r="B107" s="6" t="inlineStr">
+        <is>
+          <t>0106</t>
+        </is>
+      </c>
+      <c r="C107" s="6" t="inlineStr">
+        <is>
+          <t>TRC-22-HW1-B-0106</t>
+        </is>
+      </c>
+      <c r="D107" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-23T21:20:00Z</t>
+        </is>
+      </c>
+      <c r="E107" s="6" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="F107" s="6" t="inlineStr">
+        <is>
+          <t>HW1-B</t>
+        </is>
+      </c>
+      <c r="G107" s="6" t="inlineStr">
+        <is>
+          <t>build</t>
+        </is>
+      </c>
+      <c r="H107" s="6" t="inlineStr">
+        <is>
+          <t>105</t>
+        </is>
+      </c>
+      <c r="I107" s="6" t="inlineStr">
+        <is>
+          <t>HW1 C-STORE (the projection drain is now a scheduled job under a breaker + observability)</t>
+        </is>
+      </c>
+      <c r="J107" s="6" t="inlineStr">
+        <is>
+          <t>spine</t>
+        </is>
+      </c>
+      <c r="K107" s="6" t="inlineStr">
+        <is>
+          <t>I22-HW1B-reliability</t>
+        </is>
+      </c>
+      <c r="L107" s="6" t="inlineStr">
+        <is>
+          <t>hardening/reliability-breadth</t>
+        </is>
+      </c>
+      <c r="M107" s="6" t="inlineStr">
+        <is>
+          <t>[framework v1.5] HW1 breadth: circuit-breaker + timeout for external seams (HS-03); deterministic scheduler for the outbox-&gt;projector drain + reconciliation (REC-03/HS-02, previously invoked by nothing); observability (metrics/latency/SLO); readiness=liveness (HS-06). Wired via /api/ops/health.</t>
+        </is>
+      </c>
+      <c r="N107" s="6" t="inlineStr">
+        <is>
+          <t>ha-scale.md HS-03/HS-06; reconciliation.md REC-03; the HW1 projection consumer (now driven by a real scheduled job)</t>
+        </is>
+      </c>
+      <c r="O107" s="6" t="inlineStr">
+        <is>
+          <t>src/lib/reliability/{circuitBreaker,scheduler,bootstrap,index}.ts + src/lib/observability/{context,index}.ts + src/app/api/ops/health/route.ts (GET health+SLO, POST scheduler tick) + tests. Gates: tsc 0, 5 tests pass, E14 122/122 (entries 231-&gt;232, reachable 574-&gt;581 WIRED), demo 26 pass.</t>
+        </is>
+      </c>
+      <c r="P107" s="6" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="Q107" s="6" t="inlineStr"/>
+      <c r="R107" s="6" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S107" s="6" t="inlineStr">
+        <is>
+          <t>Closes HS-03 (breaker+timeout), REC-03/HS-02 (scheduled sweep), HS-06 (liveness), observability. Deterministic (clock injected) so unit-testable; production binds the same API to a real worker + metrics backend. Demo untouched.</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="6" t="n">
+        <v>107</v>
+      </c>
+      <c r="B108" s="6" t="inlineStr">
+        <is>
+          <t>0107</t>
+        </is>
+      </c>
+      <c r="C108" s="6" t="inlineStr">
+        <is>
+          <t>TRC-23-HW2-B-0107</t>
+        </is>
+      </c>
+      <c r="D108" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-23T21:45:00Z</t>
+        </is>
+      </c>
+      <c r="E108" s="6" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="F108" s="6" t="inlineStr">
+        <is>
+          <t>HW2-B</t>
+        </is>
+      </c>
+      <c r="G108" s="6" t="inlineStr">
+        <is>
+          <t>build</t>
+        </is>
+      </c>
+      <c r="H108" s="6" t="inlineStr">
+        <is>
+          <t>105</t>
+        </is>
+      </c>
+      <c r="I108" s="6" t="inlineStr">
+        <is>
+          <t>HW2 C-AUD (disclosure is the member-facing dimension of the audit spine); HW-SEC tenant scope</t>
+        </is>
+      </c>
+      <c r="J108" s="6" t="inlineStr">
+        <is>
+          <t>spine</t>
+        </is>
+      </c>
+      <c r="K108" s="6" t="inlineStr">
+        <is>
+          <t>I23-HW2B-disclosures</t>
+        </is>
+      </c>
+      <c r="L108" s="6" t="inlineStr">
+        <is>
+          <t>hardening/compliance-breadth</t>
+        </is>
+      </c>
+      <c r="M108" s="6" t="inlineStr">
+        <is>
+          <t>[framework v1.5] HW2 breadth: HIPAA accounting-of-disclosures (AUD-10) - record who received a member's PHI, when, purpose; classify accountable vs exempt (treatment/payment/operations); enforce 6-year retention (flag purgeable, never auto-delete). Wired: FHIR break-glass records an accountable disclosure; /api/ops/disclosures returns the accounting.</t>
+        </is>
+      </c>
+      <c r="N108" s="6" t="inlineStr">
+        <is>
+          <t>audit.md AUD-10 (accounting-of-disclosures, read-audit, retention); the C-AUD tamper-evident ledger; the FHIR break-glass path</t>
+        </is>
+      </c>
+      <c r="O108" s="6" t="inlineStr">
+        <is>
+          <t>src/lib/server/disclosure.ts (DisclosureLog + isAccountable + retention + fail-closed factory) + FHIR break-glass disclosure recording + src/app/api/ops/disclosures/route.ts (tenant+authz) + tests. Gates: tsc 0, disclosure+fhir tests pass, E14 122/122 (entries 232-&gt;233, reachable 581-&gt;583 WIRED), demo 26 pass.</t>
+        </is>
+      </c>
+      <c r="P108" s="6" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="Q108" s="6" t="inlineStr"/>
+      <c r="R108" s="6" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S108" s="6" t="inlineStr">
+        <is>
+          <t>AUD-10 accounting-of-disclosures with HIPAA accountable/exempt classification + 6-year retention. PHI-safe (references+purpose only). Break-glass over a consent opt-out is correctly recorded as accountable. Demo untouched.</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="6" t="n">
+        <v>108</v>
+      </c>
+      <c r="B109" s="6" t="inlineStr">
+        <is>
+          <t>0108</t>
+        </is>
+      </c>
+      <c r="C109" s="6" t="inlineStr">
+        <is>
+          <t>TRC-24-HW-FIN-B-0108</t>
+        </is>
+      </c>
+      <c r="D109" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-23T22:05:00Z</t>
+        </is>
+      </c>
+      <c r="E109" s="6" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="F109" s="6" t="inlineStr">
+        <is>
+          <t>HW-FIN-B</t>
+        </is>
+      </c>
+      <c r="G109" s="6" t="inlineStr">
+        <is>
+          <t>build</t>
+        </is>
+      </c>
+      <c r="H109" s="6" t="inlineStr">
+        <is>
+          <t>105</t>
+        </is>
+      </c>
+      <c r="I109" s="6" t="inlineStr">
+        <is>
+          <t>HW-FIN C-SUB (the scrub feeds submittable encounters into this pipeline)</t>
+        </is>
+      </c>
+      <c r="J109" s="6" t="inlineStr">
+        <is>
+          <t>spine</t>
+        </is>
+      </c>
+      <c r="K109" s="6" t="inlineStr">
+        <is>
+          <t>I24-HWFINB-submission</t>
+        </is>
+      </c>
+      <c r="L109" s="6" t="inlineStr">
+        <is>
+          <t>hardening/financial-breadth</t>
+        </is>
+      </c>
+      <c r="M109" s="6" t="inlineStr">
+        <is>
+          <t>[framework v1.5] HW-FIN breadth: the encounter-submission pipeline (C-SUB pipeline half) - build a submission batch, reconcile against 999/277CA/MAO-002 acknowledgments (a reject at ANY level blocks acceptance), drive resubmission with attempt limits; COB order-of-benefits (MSP + Medicaid-last-resort + birthday rule). Only ACCEPTED encounters earn risk revenue.</t>
+        </is>
+      </c>
+      <c r="N109" s="6" t="inlineStr">
+        <is>
+          <t>financial-integrity.md (no encounter-submission pipeline = no risk revenue earned; COB order-of-benefits); HW-FIN C-SUB submission gate</t>
+        </is>
+      </c>
+      <c r="O109" s="6" t="inlineStr">
+        <is>
+          <t>src/lib/finance/submission/{pipeline,cob,index}.ts (buildBatch/reconcile/buildResubmission + orderOfBenefits/primaryPayer) + src/app/api/finance/submission/route.ts (build + reconcile modes, tenant+authz) + tests. Gates: tsc 0, 6 tests pass, E14 122/122 (entries 233-&gt;234, reachable 583-&gt;587 WIRED), demo 26 pass.</t>
+        </is>
+      </c>
+      <c r="P109" s="6" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="Q109" s="6" t="inlineStr"/>
+      <c r="R109" s="6" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S109" s="6" t="inlineStr">
+        <is>
+          <t>Closes the 'no risk revenue earned' Crit: nothing is earned until an encounter is ACCEPTED (no rejecting ack at 999/277CA/MAO-002). COB prevents overpayment/FWA exposure. Live X12/EDPS transport is the NS-05 ceiling; the reconciliation logic is production-real. Demo untouched.</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="6" t="n">
+        <v>109</v>
+      </c>
+      <c r="B110" s="6" t="inlineStr">
+        <is>
+          <t>0109</t>
+        </is>
+      </c>
+      <c r="C110" s="6" t="inlineStr">
+        <is>
+          <t>TRC-25-HW-AI-B-0109</t>
+        </is>
+      </c>
+      <c r="D110" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-23T22:25:00Z</t>
+        </is>
+      </c>
+      <c r="E110" s="6" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="F110" s="6" t="inlineStr">
+        <is>
+          <t>HW-AI-B</t>
+        </is>
+      </c>
+      <c r="G110" s="6" t="inlineStr">
+        <is>
+          <t>build</t>
+        </is>
+      </c>
+      <c r="H110" s="6" t="inlineStr">
+        <is>
+          <t>105</t>
+        </is>
+      </c>
+      <c r="I110" s="6" t="inlineStr">
+        <is>
+          <t>HW-AI C-DEC (fairness monitors the decisions the invariant governs)</t>
+        </is>
+      </c>
+      <c r="J110" s="6" t="inlineStr">
+        <is>
+          <t>spine</t>
+        </is>
+      </c>
+      <c r="K110" s="6" t="inlineStr">
+        <is>
+          <t>I25-HWAIB-fairness</t>
+        </is>
+      </c>
+      <c r="L110" s="6" t="inlineStr">
+        <is>
+          <t>hardening/ai-governance-breadth</t>
+        </is>
+      </c>
+      <c r="M110" s="6" t="inlineStr">
+        <is>
+          <t>[framework v1.5] HW-AI breadth: fairness/disparate-impact monitoring (the equity claim, previously ZERO tested). EEOC four-fifths rule over AI-influenced decision outcomes by PHI-safe cohort; flag a cohort whose favorable rate &lt; 80% of the reference; report only, never auto-act. Wired: the PA decision route records the cohort outcome; /api/ops/fairness reports.</t>
+        </is>
+      </c>
+      <c r="N110" s="6" t="inlineStr">
+        <is>
+          <t>ai-governance.md (zero fairness/equity testing); HW-AI C-DEC decision surface</t>
+        </is>
+      </c>
+      <c r="O110" s="6" t="inlineStr">
+        <is>
+          <t>src/lib/agents/governance/fairness.ts (aggregate + disparateImpact four-fifths + record/current) + decision-route cohort recording + src/app/api/ops/fairness/route.ts (409 when flagged) + tests. Gates: tsc 0, 4 tests pass, E14 122/122 (entries 234-&gt;235, reachable 587-&gt;589 WIRED), demo 26 pass.</t>
+        </is>
+      </c>
+      <c r="P110" s="6" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="Q110" s="6" t="inlineStr"/>
+      <c r="R110" s="6" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S110" s="6" t="inlineStr">
+        <is>
+          <t>Addresses the equity Crit with the EEOC four-fifths rule; small-sample cohorts reported but not flagged (no false alarm). PHI-safe (coarse cohort labels + counts). Reports for human review, never auto-acts on a disparity. Demo untouched.</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="6" t="n">
+        <v>110</v>
+      </c>
+      <c r="B111" s="6" t="inlineStr">
+        <is>
+          <t>0110</t>
+        </is>
+      </c>
+      <c r="C111" s="6" t="inlineStr">
+        <is>
+          <t>TRC-26-HW4-B-0110</t>
+        </is>
+      </c>
+      <c r="D111" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-23T22:45:00Z</t>
+        </is>
+      </c>
+      <c r="E111" s="6" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="F111" s="6" t="inlineStr">
+        <is>
+          <t>HW4-B</t>
+        </is>
+      </c>
+      <c r="G111" s="6" t="inlineStr">
+        <is>
+          <t>build</t>
+        </is>
+      </c>
+      <c r="H111" s="6" t="inlineStr">
+        <is>
+          <t>105</t>
+        </is>
+      </c>
+      <c r="I111" s="6" t="inlineStr">
+        <is>
+          <t>HW1 C-STORE graph + HW-SEC tenant scope; the existing authored holistic engine (mock disposition)</t>
+        </is>
+      </c>
+      <c r="J111" s="6" t="inlineStr">
+        <is>
+          <t>spine</t>
+        </is>
+      </c>
+      <c r="K111" s="6" t="inlineStr">
+        <is>
+          <t>I26-HW4B-holistic-context</t>
+        </is>
+      </c>
+      <c r="L111" s="6" t="inlineStr">
+        <is>
+          <t>hardening/whole-person-breadth</t>
+        </is>
+      </c>
+      <c r="M111" s="6" t="inlineStr">
+        <is>
+          <t>[framework v1.5] HW4 breadth: holistic-context SEAM (WPC-01/02) - the engine returned rich context only for authored demo members; the real projected graph reached no route. mock/seeded=authored engine context (demo intact, Maria et al.); production=aggregate the real projected graph via a registered aggregator, fail-closed. UI reads one interface; config chooses the source.</t>
+        </is>
+      </c>
+      <c r="N111" s="6" t="inlineStr">
+        <is>
+          <t>whole-person-care.md WPC-01/02 (empty context for non-demo members; projected graph wired to zero routes); existing holisticContextEngine.buildContext</t>
+        </is>
+      </c>
+      <c r="O111" s="6" t="inlineStr">
+        <is>
+          <t>src/lib/wpc/holisticContext.ts (resolveHolisticContext seam + fail-closed aggregator) + src/app/api/wpc/context/route.ts (tenant+authz, 503 fail-closed) + tests. Gates: tsc 0, 3 tests pass, E14 122/122 (entries 235-&gt;236, reachable 589-&gt;591 WIRED), demo 26 pass.</t>
+        </is>
+      </c>
+      <c r="P111" s="6" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="Q111" s="6" t="inlineStr"/>
+      <c r="R111" s="6" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S111" s="6" t="inlineStr">
+        <is>
+          <t>De-hardcoding the demo = ADDING the production branch, never deleting the mock (constraint #2). The projected graph now reaches a real route via the seam. Production aggregator is the NS-05 wiring step; mock preserves the demo exactly. Demo untouched.</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="6" t="n">
+        <v>111</v>
+      </c>
+      <c r="B112" s="6" t="inlineStr">
+        <is>
+          <t>0111</t>
+        </is>
+      </c>
+      <c r="C112" s="6" t="inlineStr">
+        <is>
+          <t>TRC-27-HW5-B-0111</t>
+        </is>
+      </c>
+      <c r="D112" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-23T23:05:00Z</t>
+        </is>
+      </c>
+      <c r="E112" s="6" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="F112" s="6" t="inlineStr">
+        <is>
+          <t>HW5-B</t>
+        </is>
+      </c>
+      <c r="G112" s="6" t="inlineStr">
+        <is>
+          <t>build</t>
+        </is>
+      </c>
+      <c r="H112" s="6" t="inlineStr">
+        <is>
+          <t>105</t>
+        </is>
+      </c>
+      <c r="I112" s="6" t="inlineStr">
+        <is>
+          <t>every hardening module (now property-tested for invariants, not just examples)</t>
+        </is>
+      </c>
+      <c r="J112" s="6" t="inlineStr">
+        <is>
+          <t>spine</t>
+        </is>
+      </c>
+      <c r="K112" s="6" t="inlineStr">
+        <is>
+          <t>I27-HW5B-property-tests</t>
+        </is>
+      </c>
+      <c r="L112" s="6" t="inlineStr">
+        <is>
+          <t>hardening/test-breadth</t>
+        </is>
+      </c>
+      <c r="M112" s="6" t="inlineStr">
+        <is>
+          <t>[framework v1.5] HW5 breadth: property/fuzz tests (dependency-free seeded PRNG, reproducible) asserting INVARIANTS over all inputs for the hardening logic: contentHash order-independence+sensitivity, DEQM gapCount=max(0,denom-numer), tenant-scope membership, COB medicaid-never-primary, adverse-action monotonicity, record-lifecycle unchanged-vs-correction.</t>
+        </is>
+      </c>
+      <c r="N112" s="6" t="inlineStr">
+        <is>
+          <t>testing.md T-05 (property/fuzz); the hardening modules from I12-I26</t>
+        </is>
+      </c>
+      <c r="O112" s="6" t="inlineStr">
+        <is>
+          <t>tests/property/invariants.test.ts (6 properties x 300 randomized runs = 1800 assertions, seeded mulberry32). Gates: tsc 0, 6 property tests pass, demo 26 pass, E14 122/122 unchanged (test-only).</t>
+        </is>
+      </c>
+      <c r="P112" s="6" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="Q112" s="6" t="inlineStr"/>
+      <c r="R112" s="6" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S112" s="6" t="inlineStr">
+        <is>
+          <t>Invariant-based testing complements the example-based unit tests + the E13 mutation gate: 1800 randomized assertions found no invariant violation. Deterministic seed so any future failure reproduces. Remaining HW5 breadth (contract/Inferno in CI, testcontainer concurrency, D4 load/soak, chaos) needs live infra - named in GO_LIVE_GATES.md.</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="5" t="n">
+        <v>112</v>
+      </c>
+      <c r="B113" s="5" t="inlineStr">
+        <is>
+          <t>0112</t>
+        </is>
+      </c>
+      <c r="C113" s="5" t="inlineStr">
+        <is>
+          <t>TRC-E13-FIX-fix-0112</t>
+        </is>
+      </c>
+      <c r="D113" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-24T00:10:00Z</t>
+        </is>
+      </c>
+      <c r="E113" s="5" t="inlineStr">
+        <is>
+          <t>E13-FIX</t>
+        </is>
+      </c>
+      <c r="F113" s="5" t="inlineStr">
+        <is>
+          <t>fix</t>
+        </is>
+      </c>
+      <c r="G113" s="5" t="inlineStr">
+        <is>
+          <t>fix</t>
+        </is>
+      </c>
+      <c r="H113" s="5" t="inlineStr">
+        <is>
+          <t>105</t>
+        </is>
+      </c>
+      <c r="I113" s="5" t="inlineStr">
+        <is>
+          <t>the E13 test-link tool from framework v1.4 (bug found from the owner's CI feedback, fixed same way as the E13 mutation-tool bug in HW5)</t>
+        </is>
+      </c>
+      <c r="J113" s="5" t="inlineStr">
+        <is>
+          <t>spine</t>
+        </is>
+      </c>
+      <c r="K113" s="5" t="inlineStr">
+        <is>
+          <t>E13-testlink-ratchet</t>
+        </is>
+      </c>
+      <c r="L113" s="5" t="inlineStr">
+        <is>
+          <t>framework/enforcement</t>
+        </is>
+      </c>
+      <c r="M113" s="5" t="inlineStr">
+        <is>
+          <t>Owner-reported: E13 test-coverage gate FAILS on every commit (273 modules need test linkage). Root cause: check-testlink.mjs ran WHOLE-REPO as a hard fail (a 200+ module pre-existing backlog can never pass), and matched only FILENAME stems - so a new module imported via a barrel (its symbols used, filename not) was a FALSE POSITIVE. Fix: make the check SYMBOL-AWARE (a test using any exported symbol links the module, following barrel re-exports) and a RATCHET (testlink-baseline.json freezes the backlog; only NEW untested modules fail), matching E2/E14.</t>
+        </is>
+      </c>
+      <c r="N113" s="5" t="inlineStr">
+        <is>
+          <t>check-testlink.mjs (filename-only, whole-repo hard fail); the 268-&gt;213 false-positive drop from symbol matching; the 686-module repo</t>
+        </is>
+      </c>
+      <c r="O113" s="5" t="inlineStr">
+        <is>
+          <t>check-testlink.mjs v2 (symbol-aware linkage + --baseline/--write-baseline ratchet) + testlink-baseline.json (212 known-untested backlog, frozen) + tests/demoPreservation/fingerprint.test.ts (the 1 genuinely-untested new module, now tested) + package.json check:testlink uses the baseline + CI E13 step uses the baseline. Verified: my 26 new hardening modules are all symbol-linked (0 in the baseline); ratchet passes at baseline and catches a new untested module.</t>
+        </is>
+      </c>
+      <c r="P113" s="5" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="Q113" s="5" t="inlineStr"/>
+      <c r="R113" s="5" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S113" s="5" t="inlineStr">
+        <is>
+          <t>Same pattern as the HW5 mutation-tool fix and the E14 wiring ratchet: a gate that hard-fails on a pre-existing backlog is unusable; a ratchet + a committed baseline makes every commit pass unless it ADDS untested code, while the backlog is burned down. Symbol-aware matching removes the barrel-import false positives that were failing the hardening commits. None of the new hardening modules were actually untested - they were false positives.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:S106"/>
+  <autoFilter ref="A1:S113"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -10031,7 +10668,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E106"/>
+  <dimension ref="A1:E113"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -12903,6 +13540,195 @@
         </is>
       </c>
     </row>
+    <row r="107">
+      <c r="A107" s="6" t="inlineStr">
+        <is>
+          <t>0106</t>
+        </is>
+      </c>
+      <c r="B107" s="6" t="inlineStr">
+        <is>
+          <t>TRC-22-HW1-B-0106</t>
+        </is>
+      </c>
+      <c r="C107" s="6" t="inlineStr">
+        <is>
+          <t>BUILD I22</t>
+        </is>
+      </c>
+      <c r="D107" s="6" t="inlineStr">
+        <is>
+          <t>I22-HW1B-reliability</t>
+        </is>
+      </c>
+      <c r="E107" s="6" t="inlineStr">
+        <is>
+          <t>src/lib/reliability/{circuitBreaker,scheduler,bootstrap,index}.ts + src/lib/observability/{context,index}.ts + src/app/api/ops/health/route.ts (GET health+SLO, POST scheduler tick) + tests. Gates: tsc 0, 5 tests pass, E14 122/122 (entries 231-&gt;232, reachable 574-&gt;581 WIRED), demo 26 pass.</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="6" t="inlineStr">
+        <is>
+          <t>0107</t>
+        </is>
+      </c>
+      <c r="B108" s="6" t="inlineStr">
+        <is>
+          <t>TRC-23-HW2-B-0107</t>
+        </is>
+      </c>
+      <c r="C108" s="6" t="inlineStr">
+        <is>
+          <t>BUILD I23</t>
+        </is>
+      </c>
+      <c r="D108" s="6" t="inlineStr">
+        <is>
+          <t>I23-HW2B-disclosures</t>
+        </is>
+      </c>
+      <c r="E108" s="6" t="inlineStr">
+        <is>
+          <t>src/lib/server/disclosure.ts (DisclosureLog + isAccountable + retention + fail-closed factory) + FHIR break-glass disclosure recording + src/app/api/ops/disclosures/route.ts (tenant+authz) + tests. Gates: tsc 0, disclosure+fhir tests pass, E14 122/122 (entries 232-&gt;233, reachable 581-&gt;583 WIRED), demo 26 pass.</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="6" t="inlineStr">
+        <is>
+          <t>0108</t>
+        </is>
+      </c>
+      <c r="B109" s="6" t="inlineStr">
+        <is>
+          <t>TRC-24-HW-FIN-B-0108</t>
+        </is>
+      </c>
+      <c r="C109" s="6" t="inlineStr">
+        <is>
+          <t>BUILD I24</t>
+        </is>
+      </c>
+      <c r="D109" s="6" t="inlineStr">
+        <is>
+          <t>I24-HWFINB-submission</t>
+        </is>
+      </c>
+      <c r="E109" s="6" t="inlineStr">
+        <is>
+          <t>src/lib/finance/submission/{pipeline,cob,index}.ts (buildBatch/reconcile/buildResubmission + orderOfBenefits/primaryPayer) + src/app/api/finance/submission/route.ts (build + reconcile modes, tenant+authz) + tests. Gates: tsc 0, 6 tests pass, E14 122/122 (entries 233-&gt;234, reachable 583-&gt;587 WIRED), demo 26 pass.</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="6" t="inlineStr">
+        <is>
+          <t>0109</t>
+        </is>
+      </c>
+      <c r="B110" s="6" t="inlineStr">
+        <is>
+          <t>TRC-25-HW-AI-B-0109</t>
+        </is>
+      </c>
+      <c r="C110" s="6" t="inlineStr">
+        <is>
+          <t>BUILD I25</t>
+        </is>
+      </c>
+      <c r="D110" s="6" t="inlineStr">
+        <is>
+          <t>I25-HWAIB-fairness</t>
+        </is>
+      </c>
+      <c r="E110" s="6" t="inlineStr">
+        <is>
+          <t>src/lib/agents/governance/fairness.ts (aggregate + disparateImpact four-fifths + record/current) + decision-route cohort recording + src/app/api/ops/fairness/route.ts (409 when flagged) + tests. Gates: tsc 0, 4 tests pass, E14 122/122 (entries 234-&gt;235, reachable 587-&gt;589 WIRED), demo 26 pass.</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="6" t="inlineStr">
+        <is>
+          <t>0110</t>
+        </is>
+      </c>
+      <c r="B111" s="6" t="inlineStr">
+        <is>
+          <t>TRC-26-HW4-B-0110</t>
+        </is>
+      </c>
+      <c r="C111" s="6" t="inlineStr">
+        <is>
+          <t>BUILD I26</t>
+        </is>
+      </c>
+      <c r="D111" s="6" t="inlineStr">
+        <is>
+          <t>I26-HW4B-holistic-context</t>
+        </is>
+      </c>
+      <c r="E111" s="6" t="inlineStr">
+        <is>
+          <t>src/lib/wpc/holisticContext.ts (resolveHolisticContext seam + fail-closed aggregator) + src/app/api/wpc/context/route.ts (tenant+authz, 503 fail-closed) + tests. Gates: tsc 0, 3 tests pass, E14 122/122 (entries 235-&gt;236, reachable 589-&gt;591 WIRED), demo 26 pass.</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="6" t="inlineStr">
+        <is>
+          <t>0111</t>
+        </is>
+      </c>
+      <c r="B112" s="6" t="inlineStr">
+        <is>
+          <t>TRC-27-HW5-B-0111</t>
+        </is>
+      </c>
+      <c r="C112" s="6" t="inlineStr">
+        <is>
+          <t>BUILD I27</t>
+        </is>
+      </c>
+      <c r="D112" s="6" t="inlineStr">
+        <is>
+          <t>I27-HW5B-property-tests</t>
+        </is>
+      </c>
+      <c r="E112" s="6" t="inlineStr">
+        <is>
+          <t>tests/property/invariants.test.ts (6 properties x 300 randomized runs = 1800 assertions, seeded mulberry32). Gates: tsc 0, 6 property tests pass, demo 26 pass, E14 122/122 unchanged (test-only).</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="6" t="inlineStr">
+        <is>
+          <t>0112</t>
+        </is>
+      </c>
+      <c r="B113" s="6" t="inlineStr">
+        <is>
+          <t>TRC-E13-FIX-fix-0112</t>
+        </is>
+      </c>
+      <c r="C113" s="6" t="inlineStr">
+        <is>
+          <t>BUILD IE13-FIX</t>
+        </is>
+      </c>
+      <c r="D113" s="6" t="inlineStr">
+        <is>
+          <t>E13-testlink-ratchet</t>
+        </is>
+      </c>
+      <c r="E113" s="6" t="inlineStr">
+        <is>
+          <t>check-testlink.mjs v2 (symbol-aware linkage + --baseline/--write-baseline ratchet) + testlink-baseline.json (212 known-untested backlog, frozen) + tests/demoPreservation/fingerprint.test.ts (the 1 genuinely-untested new module, now tested) + package.json check:testlink uses the baseline + CI E13 step uses the baseline. Verified: my 26 new hardening modules are all symbol-linked (0 in the baseline); ratchet passes at baseline and catches a new untested module.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>